<commit_message>
[SCRUM-1267] Corrige R-09: Dispatch tambien se conecta como postgres con BYPASSRLS
- El primer intento con DISPATCH_DB_CONNECTION fallo por un error de QA al interpretar las comillas
  de la cadena Npgsql, no por la credencial. Dispatch si accede a la base: 1074-01 asigna la solicitud.
- Consulta de solo lectura repetida con la cadena bien interpretada (dispatch_rol_20261020T232719Z.txt):
  current_user = postgres, rolbypassrls = t.
- Reporte y matriz actualizados; se retira el pendiente de confirmar las credenciales de Dispatch.
</commit_message>
<xml_diff>
--- a/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
+++ b/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
@@ -21455,7 +21455,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Core se conecta como postgres (current_user = postgres, rolbypassrls = t). La cadena de Dispatch usa el mismo rol postgres; la conexión de solo lectura con esa cadena desde la VM fue rechazada por autenticación, así que el rol de Dispatch sale de la configuración y no de una sesión. mani_core_svc y mani_dispatch_svc: rolcanlogin = f, rolbypassrls = f.</t>
+          <t>Core y Dispatch se conectan como postgres (current_user = postgres, rolbypassrls = t), cada uno con su cadena de .env.qa. mani_core_svc y mani_dispatch_svc: rolcanlogin = f, rolbypassrls = f.</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -21465,7 +21465,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuarios de conexión)</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuario de Core); qa/regresion_sprint4/evidencia/dispatch_rol_20261020T232719Z.txt (usuario de Dispatch)</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -21475,7 +21475,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Alta (Core); Media (Dispatch)</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
[SCRUM-1267] Registra la primera corrida del gate de CI desde el runner de Calidad
- Gate habilitado en MANI-APIGateway (environment qa-regresion, secreto QA_JWT_SECRET y variables QA_*)
  y ejecutado desde nbig02-calidad (run 39513870492): Newman 20261020T234635Z (77 solicitudes, 125
  aserciones, 5 fallidas) y Playwright 20261020T235520Z (11 pruebas, 9 aprobadas). Los dos jobs quedan en
  rojo por R-01 a R-04, con el mismo resultado que en la VM de QA.
- Evidencia versionada desde los artefactos del run, revisada sin credenciales.
- L-02 cerrada, L-08 y DoD de SCRUM-1277 y SCRUM-1278 actualizados.
</commit_message>
<xml_diff>
--- a/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
+++ b/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
@@ -22149,17 +22149,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Punto de ejecución</t>
+          <t>Punto de ejecución (cerrada)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Newman y Playwright se ejecutaron dentro de la VM de QA (localhost), no desde el runner de Calidad que prevé la guía CFG4-03. El puerto 80 de QA desde el equipo del QA por la VPN responde reset; no se probó desde Calidad.</t>
+          <t>Cerrada el 20 de octubre: además de la VM de QA, la regresión corrió desde el runner nbig02-calidad de la VM de Calidad (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)) con el mismo resultado. Desde el equipo del QA por la VPN, el puerto 80 de QA sigue respondiendo reset.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -22316,7 +22316,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>El workflow qa-regresion.yml no se ha ejecutado. Según GOBIERNO_DEL_EQUIPO §2.3, CI/CD y secretos los decide DevOps: el environment, el secreto y las variables quedan como propuesta para DevOps.</t>
+          <t>Habilitado por QA el 20 de octubre y ejecutado una vez (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 77 solicitudes, 125 aserciones y 5 fallidas; Playwright 11 pruebas y 9 aprobadas. Los dos jobs quedan en rojo por R-01 a R-04 (corrida en rojo del DoD); la corrida en verde depende de esas correcciones. No es check obligatorio de la rama. GOBIERNO_DEL_EQUIPO §2.3 asigna CI/CD y secretos a DevOps.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -22326,7 +22326,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>QA y DevOps</t>
         </is>
       </c>
     </row>
@@ -22649,7 +22649,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Vigentes: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida). Anteriores: Newman 20261020T212453Z y Playwright 20261020T212519Z. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z.</t>
+          <t>Vigentes: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida). Anteriores: Newman 20261020T212453Z y Playwright 20261020T212519Z. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z. Gate de CI desde el runner de Calidad (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 20261020T234635Z y Playwright 20261020T235520Z.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[SCRUM-1267] Registra en el reporte y la matriz los defectos creados en Jira (SCRUM-1358 a SCRUM-1362)
</commit_message>
<xml_diff>
--- a/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
+++ b/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
@@ -20788,12 +20788,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>BUG-SEC-04 (ya propuesto en SCRUM-1266, D-02)</t>
+          <t>BUG-SEC-04 - registrado como SCRUM-1362 (20 oct)</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto en Jira</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -20890,12 +20890,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>BUG-QA-07</t>
+          <t>BUG-QA-07 - registrado como SCRUM-1361 (20 oct)</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto en Jira</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -21094,12 +21094,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>BUG-GW-01</t>
+          <t>BUG-GW-01 - registrado como SCRUM-1359 (20 oct)</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto en Jira</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -21196,12 +21196,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>BUG-CORE-01</t>
+          <t>BUG-CORE-01 - registrado como SCRUM-1358 (20 oct)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto en Jira</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -21298,12 +21298,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>BUG-CORE-02</t>
+          <t>BUG-CORE-02 - registrado como SCRUM-1360 (20 oct)</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto en Jira</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
[SCRUM-1267] Registra la validacion en QA de las correcciones de la regresion del Sprint 4
- R-01, R-02, R-03 y R-10 corregidos (MANI-APIGateway#20, MANI-Node#49, #50 y #52, MANI-.NET#11 y #13),
  promovidos a release y verificados en QA el 21 de octubre. R-04 mitigado en QA con el montaje de
  flutter.env.qa en flutter-web; la correccion en MANI-Flutter sigue pendiente.
- Corridas desde release f042817: Newman 20261021T161015Z (77 solicitudes, 125 aserciones, 0 fallidas) y
  Playwright 20261021T170129Z (11 de 11). Login real con ES256 verificado y tokens ES256 falsificados
  rechazados. R-06, R-07, R-09 y R-11 reverificados sin cambios.
- Estados: 853, 856 y 1066 pasan a Ejecutado y 1060 a Sin ejecutar; multi-tenant 10 aprobados, 5
  bloqueados y 75 sin ejecutar. Matriz, limites, pendientes y DoD actualizados.
- Corrige inconsistencias: lineas citadas en R-01 y R-02, DoD de defectos y discrepancias con Jira.
</commit_message>
<xml_diff>
--- a/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
+++ b/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'defectos_propuestos'!$A$1:$T$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'equivalencias'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'limitaciones'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'criterios'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'criterios'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ambiente'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -752,12 +752,12 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -860,12 +860,12 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -945,24 +945,24 @@
         <v>4</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>El aliado con el servicio asignado recibe 403 al leer las reglas del sitio (R-02); el negativo con un aliado sin asignación pasa.</t>
+          <t>El aliado asignado ya lee las reglas del sitio (853-04 en 200 desde el 21 oct, R-02 corregido por MANI-Node#50 y MANI-.NET#11); el aliado sin asignación sigue recibiendo 403 y el de otro tenant 404.</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>R-02, R-10, R-04</t>
+          <t>R-02 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1277,24 +1277,24 @@
         <v>6</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>856-02 (no concluyente)</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>Los documentos legales no se pueden consultar antes del registro (R-01, 856-05). El rechazo del consentimiento sobre un documento de t2 (856-03, LEGAL_DOCUMENT_NOT_FOUND) y la no duplicación del consentimiento (856-06) aprueban en la corrida 20261020T224842Z. 856-02 sigue no concluyente (el cliente t1 ya había consentido). Core no expone una consulta del consentimiento propio (C4 de SCRUM-1257): por confirmar con Desarrollo. Casos que no cuentan: 856-02 (no concluyente).</t>
+          <t>Los documentos legales ya se consultan sin token (856-05 en 200 desde el 21 oct, R-01 corregido por MANI-APIGateway#20). El consentimiento sobre un documento de t2 se rechaza con LEGAL_DOCUMENT_NOT_FOUND (856-03) y repetirlo no lo duplica (856-06). 856-02 sigue no concluyente. Core no expone una consulta del consentimiento propio (C4): por confirmar con Desarrollo. Casos que no cuentan: 856-02 (no concluyente).</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>R-01, R-10, R-04</t>
+          <t>R-01 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1416,12 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-11</t>
+          <t>R-10 (corregido), R-11</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1640,12 +1640,12 @@
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-11</t>
+          <t>R-10 (corregido), R-11</t>
         </is>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2707,14 +2707,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>Bloqueado</t>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Sin ejecutar</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>Historia de interfaz (datasource de Flutter). La web de QA usa el Supabase de producción y localhost (R-04) y un usuario real no puede usar rutas protegidas (R-10). Los casos API previstos para esta historia no se ejecutaron (cobertura de QA).</t>
+          <t>Historia de interfaz. Desde el 21 oct ya no la bloquean R-04 (mitigado en QA) ni R-10 (corregido), pero QA no ha ejecutado sus casos de interfaz ni los de API por el Gateway (CC-2 a CC-4 y X1 a X6). "Sin ejecutar" no es un estado del vocabulario de SCRUM-1267: se declara para no ocultar la brecha.</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="W20" s="2" t="inlineStr">
         <is>
-          <t>R-04, R-10</t>
+          <t>R-04 (mitigado en QA), R-10 (corregido)</t>
         </is>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>DevOps (R-04) y Desarrollo de Core (R-10); QA en la cobertura API</t>
+          <t>QA (casos de interfaz y de API sin ejecutar)</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2832,12 +2832,12 @@
       </c>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2940,12 +2940,12 @@
       </c>
       <c r="W22" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3052,12 @@
       </c>
       <c r="W23" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04, R-11</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA), R-11</t>
         </is>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="Z23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3164,12 @@
       </c>
       <c r="W24" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04, R-11</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA), R-11</t>
         </is>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3384,12 @@
       </c>
       <c r="W26" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3469,39 +3469,39 @@
         <v>3</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>Listado y detalle de verificación responden 500 por documento_kyc.created_at (R-03); aprobar, rechazar y auditoría no se pudieron ejecutar.</t>
+          <t>Listado y detalle de verificación responden 200 desde el 21 oct (R-03 corregido por MANI-Node#49). Aprobar, rechazar, auditoría (T10) y el X6 de Storage siguen sin ejecutar.</t>
         </is>
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>X1 aprobado; X2 sin ejecutar; X3 sin ejecutar; X4 sin ejecutar; X5 sin ejecutar; X6 bloqueado (R-03)</t>
+          <t>X1 aprobado; X2 sin ejecutar; X3 sin ejecutar; X4 sin ejecutar; X5 sin ejecutar; X6 sin ejecutar</t>
         </is>
       </c>
       <c r="W27" s="2" t="inlineStr">
         <is>
-          <t>R-03, R-10, R-04</t>
+          <t>R-03 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y27" s="2" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Fallido</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>Fallido</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -16821,7 +16821,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16863,7 +16863,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16905,7 +16905,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16947,7 +16947,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16989,7 +16989,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17031,7 +17031,7 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17073,7 +17073,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17115,7 +17115,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17157,7 +17157,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17199,7 +17199,7 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17241,7 +17241,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17283,7 +17283,7 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17325,7 +17325,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17367,7 +17367,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17409,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17451,7 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17493,7 +17493,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17535,7 +17535,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17577,7 +17577,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17619,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17661,7 +17661,7 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17703,7 +17703,7 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17745,7 +17745,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17787,7 +17787,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17829,7 +17829,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17871,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17913,7 +17913,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17955,7 +17955,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17997,7 +17997,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18039,7 +18039,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18081,7 +18081,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18123,7 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18165,7 +18165,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18207,7 +18207,7 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18249,7 +18249,7 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18291,7 +18291,7 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18333,7 +18333,7 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18375,7 +18375,7 @@
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18421,7 +18421,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18463,7 +18463,7 @@
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18489,16 +18489,16 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>401</v>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>R-01</t>
+          <t>R-01 (corregido)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -18506,10 +18506,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-01 corregido por MANI-APIGateway#20; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18555,7 +18559,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18601,7 +18605,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18651,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18689,7 +18693,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18731,7 +18735,7 @@
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18773,7 +18777,7 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18815,7 +18819,7 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18857,7 +18861,7 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18899,7 +18903,7 @@
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18941,7 +18945,7 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18983,7 +18987,7 @@
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19025,7 +19029,7 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19067,7 +19071,7 @@
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19113,7 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19151,7 +19155,7 @@
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19177,16 +19181,16 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>R-03</t>
+          <t>R-03 (corregido)</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -19194,10 +19198,14 @@
           <t>US0213M2-P1 (completo)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-03 corregido por MANI-Node#49; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19223,16 +19231,16 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>R-03</t>
+          <t>R-03 (corregido)</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -19240,10 +19248,14 @@
           <t>US0213M2-P1 (parcial)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-03 corregido por MANI-Node#49; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19285,7 +19297,7 @@
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19331,7 +19343,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19373,7 +19385,7 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19415,7 +19427,7 @@
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19457,7 +19469,7 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19499,7 +19511,7 @@
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19541,7 +19553,7 @@
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19583,7 +19595,7 @@
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19625,7 +19637,7 @@
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19667,7 +19679,7 @@
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19709,7 +19721,7 @@
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19751,7 +19763,7 @@
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19793,7 +19805,7 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19835,7 +19847,7 @@
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19889,7 @@
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19919,7 +19931,7 @@
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19945,16 +19957,16 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>403</v>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R-02</t>
+          <t>R-02 (corregido)</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -19962,10 +19974,14 @@
           <t>US0223-P1 (parcial)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-02 corregido por MANI-Node#50 y MANI-.NET#11; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20103,7 +20119,7 @@
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20145,7 +20161,7 @@
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20189,7 +20205,7 @@
       <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20233,7 +20249,7 @@
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20277,7 +20293,7 @@
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20321,7 +20337,7 @@
       <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20365,7 +20381,7 @@
       <c r="I85" s="2" t="inlineStr"/>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20409,7 +20425,7 @@
       <c r="I86" s="2" t="inlineStr"/>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20439,14 +20455,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -20454,10 +20470,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-04 mitigado en QA: /opt/mani monta flutter.env.qa en assets/.env; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20487,14 +20507,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -20502,10 +20522,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-04 mitigado en QA: /opt/mani monta flutter.env.qa en assets/.env; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20549,7 +20573,7 @@
       <c r="I89" s="2" t="inlineStr"/>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20593,7 +20617,7 @@
       <c r="I90" s="2" t="inlineStr"/>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20637,7 +20661,7 @@
       <c r="I91" s="2" t="inlineStr"/>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20793,7 +20817,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -20853,7 +20877,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>MANI-docs qa/monitoreo_qas/evidencia/20261020T020546Z_d02/confirmacion_d02_login_real.txt; MANI-Node release src/routes/auth.routes.js:9 (ALLOWED_ALGORITHMS = HS256)</t>
+          <t>MANI-docs qa/monitoreo_qas/evidencia/20261020T020546Z_d02/confirmacion_d02_login_real.txt; MANI-Node release src/routes/auth.routes.js:9 (ALLOWED_ALGORITHMS = HS256). Verificación del 21 oct: MANI-Node#52 y MANI-.NET#13 (develop); MANI-Node#53 y MANI-.NET#14 (release). Login real ES256 con 200 (login_real_es256_20261021T164543Z.txt) y tokens ES256 falsificados con 401 (es256_negativos_20261021.txt). ADR-0031 en MANI-docs#59, abierto.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -20895,7 +20919,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Mitigado en QA (21 oct); corrección en el repositorio pendiente</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -20955,7 +20979,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>playwright_resultados.json; flutter_login_qa.png; MANI-Flutter release .github/workflows/docker-publish.yml:30</t>
+          <t>playwright_resultados.json; flutter_login_qa.png; MANI-Flutter release .github/workflows/docker-publish.yml:30. Verificación del 21 oct: En /opt/mani se monta flutter.env.qa en assets/.env (cambio manual, sin versionar). Playwright FW-02 y FW-03 aprueban (playwright_resultados_20261021T170129Z.json). MANI-Flutter sigue copiando .env.example al construir la imagen.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -21057,7 +21081,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Sin evidencia versionada</t>
+          <t>Sin evidencia versionada. Verificación del 21 oct: El 21 oct se sumó el montaje manual de flutter.env.qa (R-04) al compose sin versionar de /opt/mani.</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -21099,7 +21123,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -21159,7 +21183,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release src/routes/legal.routes.js:7; nginx.conf sin la ruta</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release src/routes/legal.routes.js:8; nginx.conf sin la ruta. Verificación del 21 oct: MANI-APIGateway#20 (develop) y #21 (release). Newman 856-05 en 200 (newman_resumen_20261021T161015Z.json).</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -21201,7 +21225,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -21261,7 +21285,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release GetSiteRulesForAllyUseCase.js:8</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release GetSiteRulesForAllyUseCase.js:45-51. Verificación del 21 oct: MANI-Node#50 y MANI-.NET#11 (develop); MANI-Node#51 y MANI-.NET#12 (release). Newman 853-04 en 200.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -21303,7 +21327,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -21363,7 +21387,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release SupabaseDocumentoKycRepository.js:44</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release SupabaseDocumentoKycRepository.js:44. Verificación del 21 oct: MANI-Node#49 (develop) y #51 (release). Newman 1066-01 y 1066-02 en 200.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -21405,7 +21429,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -21465,7 +21489,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuario de Core); qa/regresion_sprint4/evidencia/dispatch_rol_20261020T232719Z.txt (usuario de Dispatch)</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuario de Core); qa/regresion_sprint4/evidencia/dispatch_rol_20261020T232719Z.txt (usuario de Dispatch). Verificación del 21 oct: consultas_rls_20261021T170441Z.txt (Core y Dispatch)</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -21507,7 +21531,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -21567,7 +21591,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>newman_reporte_redactado_20261020T224842Z.json (cuerpos de 862-02, 1074-03 y 1074-04; igual en newman_reporte_redactado.json de 20261020T212453Z)</t>
+          <t>newman_reporte_redactado_20261020T224842Z.json (cuerpos de 862-02, 1074-03 y 1074-04; igual en newman_reporte_redactado.json de 20261020T212453Z). Verificación del 21 oct: Cuerpos de 862-02 y 1074-04 en newman_reporte_redactado_20261021T161015Z.json</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -21609,7 +21633,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -21669,7 +21693,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (secciones 1, 1b y 1c)</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (secciones 1, 1b y 1c). Verificación del 21 oct: consultas_rls_20261021T170441Z.txt</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -21711,7 +21735,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -21771,7 +21795,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 2); qa/regresion_sprint4/evidencia/verify_0007_rls_20261020T202905Z.log</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 2); qa/regresion_sprint4/evidencia/verify_0007_rls_20261020T202905Z.log. Verificación del 21 oct: consultas_rls_20261021T170441Z.txt</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -22127,17 +22151,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Toda la regresión usó tokens HS256 sintéticos firmados con el JWT secret legado de MANI-QA. Un usuario real recibe un token ES256 que el Gateway rechaza (R-10, comprobado en SCRUM-1266). Los usuarios de prueba que SCRUM-1269 prevé no se pueden usar mientras R-10 siga abierto.</t>
+          <t>La regresión sigue usando tokens HS256 sintéticos, válidos mientras la clave HS256 legada de MANI-QA no se revoque. Desde el 21 oct un usuario real sí usa las rutas protegidas (R-10 corregido): login de admin.t1 con token ES256 y 200 en Core y Rules; Dispatch acepta el token (login_real_es256_20261021T164543Z.txt). Solo se verificó con ese usuario y esas tres rutas.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo (R-10)</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22208,7 +22232,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>No se ejecutaron flujos de interfaz: la web de QA usa el Supabase de producción (R-04) y, aunque se corrija, un usuario real no puede usar rutas protegidas (R-10).</t>
+          <t>No se ejecutaron flujos de interfaz. Desde el 21 oct R-04 está mitigado en QA y R-10 corregido, así que ya no los bloquean: la suite Playwright no tiene todavía flujos Flutter Web → Gateway → servicios.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -22218,7 +22242,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>DevOps y Desarrollo</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22235,7 +22259,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>B4-01 borra una ausencia inexistente y solo es un control; el borrado ajeno se prueba en 855-04. B6 se ejecutó sobre el detalle de verificación de otro tenant; las URL firmadas de Storage no se probaron (R-03).</t>
+          <t>B4-01 es un control con un id inexistente; el borrado ajeno se prueba en 855-04. B6 no cubre las URL firmadas de Storage: R-03, que lo impedía, está corregido desde el 21 oct, pero el caso no se ha ejecutado.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -22245,7 +22269,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Prueba de QA</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22316,7 +22340,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Habilitado por QA el 20 de octubre y ejecutado una vez (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 77 solicitudes, 125 aserciones y 5 fallidas; Playwright 11 pruebas y 9 aprobadas. Los dos jobs quedan en rojo por R-01 a R-04 (corrida en rojo del DoD); la corrida en verde depende de esas correcciones. No es check obligatorio de la rama. GOBIERNO_DEL_EQUIPO §2.3 asigna CI/CD y secretos a DevOps.</t>
+          <t>Habilitado por QA el 20 oct y ejecutado en CI una vez (run 39513870492), en rojo por R-01 a R-04 (corrida en rojo del DoD). Tras las correcciones, la regresión del 21 oct en la VM de QA da 0 fallas (Newman 20261021T161015Z y Playwright 20261021T170129Z), pero la corrida en verde en CI no se ha hecho. El gate no es un check obligatorio de la rama. GOBIERNO_DEL_EQUIPO §2.3 asigna CI/CD y secretos a DevOps.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -22343,7 +22367,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>RLS no se ejerce en QA (R-06, R-07 y R-09, con evidencia en consultas_rls_20261020T225146Z.txt). El aislamiento comprobado es el de la aplicación a través del Gateway.</t>
+          <t>RLS no se ejerce en QA (R-06, R-07 y R-09, reverificados el 21 oct en consultas_rls_20261021T170441Z.txt). El aislamiento comprobado es el de la aplicación a través del Gateway.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -22423,7 +22447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22505,53 +22529,65 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Multi-tenant X1 a X6 (SCRUM-1279)</t>
+          <t>Sin ejecutar (historia)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Por caso: aprobado, fallido, bloqueado o no ejecutable, según el DoD de SCRUM-1279; "no aplica" cuando SCRUM-1264 lo declara así y "sin ejecutar" cuando el caso es ejecutable y QA no lo corrió. "(parcial)" indica que el caso de regresión cubre una parte del caso diseñado.</t>
+          <t>La historia ya no tiene bloqueo externo y QA no ha ejecutado sus casos. No es un estado del vocabulario de SCRUM-1267: se declara para no ocultar la brecha (usado en SCRUM-1060 desde el 21 de octubre).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Cobertura de un caso de SCRUM-1264</t>
+          <t>Multi-tenant X1 a X6 (SCRUM-1279)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>completo: un caso válido verifica lo que pide el caso diseñado; parcial: verifica una parte; sin ejecutar: ningún caso válido lo cubre.</t>
+          <t>Por caso: aprobado, fallido, bloqueado o no ejecutable, según el DoD de SCRUM-1279; "no aplica" cuando SCRUM-1264 lo declara así y "sin ejecutar" cuando el caso es ejecutable y QA no lo corrió. "(parcial)" indica que el caso de regresión cubre una parte del caso diseñado.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Caso no válido, no concluyente o excluido</t>
+          <t>Cobertura de un caso de SCRUM-1264</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>No cuenta como evidencia (ver la nota del caso).</t>
+          <t>completo: un caso válido verifica lo que pide el caso diseñado; parcial: verifica una parte; sin ejecutar: ningún caso válido lo cubre.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Caso no válido, no concluyente o excluido</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>No cuenta como evidencia (ver la nota del caso).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Origen</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Desarrollo: la prueba sigue el criterio o el contrato y el sistema responde distinto. DevOps: el mismo código funciona con otra configuración o falta un componente del despliegue. QA: la prueba, los datos o la cobertura no corresponden al criterio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22589,7 +22625,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-20 (regresión) y 2026-10-21 (validación de las correcciones)</t>
         </is>
       </c>
     </row>
@@ -22601,7 +22637,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>QA 10.43.100.141 (release; Gateway 82473d6, Core 2745bb0, Rules e90f32b, Dispatch 41ba171, Flutter 74bab53, Landing a82b94e; base Supabase MANI-QA)</t>
+          <t>QA 10.43.100.141, rama release, base Supabase MANI-QA. Desde el redespliegue del 21 oct: Gateway f042817, Core 8ad4a35, Rules e90f32b, Dispatch 0998a3d, Flutter 8e606e4 y Landing a82b94e, iguales a la cabeza de release (ambiente_qa_20261021.txt). El 20 oct: Gateway 82473d6, Core 2745bb0, Dispatch 41ba171 y Flutter 74bab53.</t>
         </is>
       </c>
     </row>
@@ -22625,7 +22661,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tokens HS256 sintéticos firmados en la VM con el JWT secret legado de MANI-QA (L-01, R-10)</t>
+          <t>Tokens HS256 sintéticos firmados en la VM con el JWT secret legado de MANI-QA (L-01). Desde el 21 oct, login real con ES256 verificado para admin.t1 (R-10 corregido).</t>
         </is>
       </c>
     </row>
@@ -22637,7 +22673,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Compose, .env.qa y recreación de contenedores: QA (Santiago Hernández). Migraciones de Core 0001-0010 y 0013 aplicadas por QA desde el SQL Editor de MANI-QA. Respaldo previo en /opt/mani. Según GOBIERNO_DEL_EQUIPO §2.3 estas decisiones corresponden a DevOps; comunicación formal a DevOps pendiente.</t>
+          <t>Compose, .env.qa y recreación de contenedores: QA (Santiago Hernández). Migraciones de Core 0001-0010 y 0013 aplicadas por QA desde el SQL Editor de MANI-QA. Respaldo previo en /opt/mani. Según GOBIERNO_DEL_EQUIPO §2.3 estas decisiones corresponden a DevOps; comunicación formal a DevOps pendiente. El 21 oct, QA agregó al compose de /opt/mani el montaje de flutter.env.qa en assets/.env de flutter-web (R-04, con autorización de Santiago Hernández y respaldo previo); queda para que DevOps lo valide en el despliegue.</t>
         </is>
       </c>
     </row>
@@ -22649,7 +22685,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Vigentes: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida). Anteriores: Newman 20261020T212453Z y Playwright 20261020T212519Z. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z. Gate de CI desde el runner de Calidad (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 20261020T234635Z y Playwright 20261020T235520Z.</t>
+          <t>Vigentes (21 oct, tras las correcciones): Newman 20261021T161015Z y Playwright 20261021T170129Z. Del 20 oct: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida), Newman 20261020T212453Z y Playwright 20261020T212519Z (primera corrida) y gate de CI run 39513870492. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z y 20261021T170441Z.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[SCRUM-1267] Registra la validacion en QA de las correcciones de la regresion del Sprint 4 (#60)
- R-01, R-02, R-03 y R-10 corregidos (MANI-APIGateway#20, MANI-Node#49, #50 y #52, MANI-.NET#11 y #13),
  promovidos a release y verificados en QA el 21 de octubre. R-04 mitigado en QA con el montaje de
  flutter.env.qa en flutter-web; la correccion en MANI-Flutter sigue pendiente.
- Corridas desde release f042817: Newman 20261021T161015Z (77 solicitudes, 125 aserciones, 0 fallidas) y
  Playwright 20261021T170129Z (11 de 11). Login real con ES256 verificado y tokens ES256 falsificados
  rechazados. R-06, R-07, R-09 y R-11 reverificados sin cambios.
- Estados: 853, 856 y 1066 pasan a Ejecutado y 1060 a Sin ejecutar; multi-tenant 10 aprobados, 5
  bloqueados y 75 sin ejecutar. Matriz, limites, pendientes y DoD actualizados.
- Corrige inconsistencias: lineas citadas en R-01 y R-02, DoD de defectos y discrepancias con Jira.
</commit_message>
<xml_diff>
--- a/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
+++ b/product/MANI_Matriz_Ejecucion_Sprint4.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'defectos_propuestos'!$A$1:$T$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'equivalencias'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'limitaciones'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'criterios'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'criterios'!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ambiente'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -752,12 +752,12 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -767,7 +767,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -860,12 +860,12 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -945,24 +945,24 @@
         <v>4</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>El aliado con el servicio asignado recibe 403 al leer las reglas del sitio (R-02); el negativo con un aliado sin asignación pasa.</t>
+          <t>El aliado asignado ya lee las reglas del sitio (853-04 en 200 desde el 21 oct, R-02 corregido por MANI-Node#50 y MANI-.NET#11); el aliado sin asignación sigue recibiendo 403 y el de otro tenant 404.</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>R-02, R-10, R-04</t>
+          <t>R-02 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1192,12 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1277,24 +1277,24 @@
         <v>6</v>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>856-02 (no concluyente)</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>Los documentos legales no se pueden consultar antes del registro (R-01, 856-05). El rechazo del consentimiento sobre un documento de t2 (856-03, LEGAL_DOCUMENT_NOT_FOUND) y la no duplicación del consentimiento (856-06) aprueban en la corrida 20261020T224842Z. 856-02 sigue no concluyente (el cliente t1 ya había consentido). Core no expone una consulta del consentimiento propio (C4 de SCRUM-1257): por confirmar con Desarrollo. Casos que no cuentan: 856-02 (no concluyente).</t>
+          <t>Los documentos legales ya se consultan sin token (856-05 en 200 desde el 21 oct, R-01 corregido por MANI-APIGateway#20). El consentimiento sobre un documento de t2 se rechaza con LEGAL_DOCUMENT_NOT_FOUND (856-03) y repetirlo no lo duplica (856-06). 856-02 sigue no concluyente. Core no expone una consulta del consentimiento propio (C4): por confirmar con Desarrollo. Casos que no cuentan: 856-02 (no concluyente).</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>R-01, R-10, R-04</t>
+          <t>R-01 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1416,12 +1416,12 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10 (corregido)</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-11</t>
+          <t>R-10 (corregido), R-11</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1640,12 +1640,12 @@
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-11</t>
+          <t>R-10 (corregido), R-11</t>
         </is>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2627,7 +2627,7 @@
       </c>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2707,14 +2707,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="T20" s="6" t="inlineStr">
-        <is>
-          <t>Bloqueado</t>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Sin ejecutar</t>
         </is>
       </c>
       <c r="U20" s="2" t="inlineStr">
         <is>
-          <t>Historia de interfaz (datasource de Flutter). La web de QA usa el Supabase de producción y localhost (R-04) y un usuario real no puede usar rutas protegidas (R-10). Los casos API previstos para esta historia no se ejecutaron (cobertura de QA).</t>
+          <t>Historia de interfaz. Desde el 21 oct ya no la bloquean R-04 (mitigado en QA) ni R-10 (corregido), pero QA no ha ejecutado sus casos de interfaz ni los de API por el Gateway (CC-2 a CC-4 y X1 a X6). "Sin ejecutar" no es un estado del vocabulario de SCRUM-1267: se declara para no ocultar la brecha.</t>
         </is>
       </c>
       <c r="V20" s="2" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="W20" s="2" t="inlineStr">
         <is>
-          <t>R-04, R-10</t>
+          <t>R-04 (mitigado en QA), R-10 (corregido)</t>
         </is>
       </c>
       <c r="X20" s="2" t="inlineStr">
         <is>
-          <t>DevOps (R-04) y Desarrollo de Core (R-10); QA en la cobertura API</t>
+          <t>QA (casos de interfaz y de API sin ejecutar)</t>
         </is>
       </c>
       <c r="Y20" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="Z20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2832,12 +2832,12 @@
       </c>
       <c r="W21" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y21" s="2" t="inlineStr">
@@ -2847,7 +2847,7 @@
       </c>
       <c r="Z21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2940,12 +2940,12 @@
       </c>
       <c r="W22" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y22" s="2" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="Z22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3052,12 +3052,12 @@
       </c>
       <c r="W23" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04, R-11</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA), R-11</t>
         </is>
       </c>
       <c r="X23" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y23" s="2" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="Z23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3164,12 +3164,12 @@
       </c>
       <c r="W24" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04, R-11</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA), R-11</t>
         </is>
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="Z24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3287,7 +3287,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3384,12 @@
       </c>
       <c r="W26" s="2" t="inlineStr">
         <is>
-          <t>R-10, R-04</t>
+          <t>R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>QA (cobertura de casos diseñados); Core (identidad real: R-10); DevOps y Core (interfaz: R-04, R-10)</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y26" s="2" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3469,39 +3469,39 @@
         <v>3</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>Ejecutado</t>
         </is>
       </c>
       <c r="U27" s="2" t="inlineStr">
         <is>
-          <t>Listado y detalle de verificación responden 500 por documento_kyc.created_at (R-03); aprobar, rechazar y auditoría no se pudieron ejecutar.</t>
+          <t>Listado y detalle de verificación responden 200 desde el 21 oct (R-03 corregido por MANI-Node#49). Aprobar, rechazar, auditoría (T10) y el X6 de Storage siguen sin ejecutar.</t>
         </is>
       </c>
       <c r="V27" s="2" t="inlineStr">
         <is>
-          <t>X1 aprobado; X2 sin ejecutar; X3 sin ejecutar; X4 sin ejecutar; X5 sin ejecutar; X6 bloqueado (R-03)</t>
+          <t>X1 aprobado; X2 sin ejecutar; X3 sin ejecutar; X4 sin ejecutar; X5 sin ejecutar; X6 sin ejecutar</t>
         </is>
       </c>
       <c r="W27" s="2" t="inlineStr">
         <is>
-          <t>R-03, R-10, R-04</t>
+          <t>R-03 (corregido), R-10 (corregido), R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="X27" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo</t>
+          <t>QA (cobertura de casos diseñados)</t>
         </is>
       </c>
       <c r="Y27" s="2" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="Z28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Fallido</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>Fallido</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -16821,7 +16821,7 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16863,7 +16863,7 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16905,7 +16905,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16947,7 +16947,7 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -16989,7 +16989,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17031,7 +17031,7 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17073,7 +17073,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17115,7 +17115,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17157,7 +17157,7 @@
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17199,7 +17199,7 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17241,7 +17241,7 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17283,7 +17283,7 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17325,7 +17325,7 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17367,7 +17367,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17409,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17451,7 @@
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17493,7 +17493,7 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17535,7 +17535,7 @@
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17577,7 +17577,7 @@
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17619,7 +17619,7 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17661,7 +17661,7 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17703,7 +17703,7 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17745,7 +17745,7 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17787,7 +17787,7 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17829,7 +17829,7 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17871,7 +17871,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17913,7 +17913,7 @@
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17955,7 +17955,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -17997,7 +17997,7 @@
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18039,7 +18039,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18081,7 +18081,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18123,7 +18123,7 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18165,7 +18165,7 @@
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18207,7 +18207,7 @@
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18249,7 +18249,7 @@
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18291,7 +18291,7 @@
       <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18333,7 +18333,7 @@
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18375,7 +18375,7 @@
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18421,7 +18421,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18463,7 +18463,7 @@
       <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18489,16 +18489,16 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>401</v>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>R-01</t>
+          <t>R-01 (corregido)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -18506,10 +18506,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-01 corregido por MANI-APIGateway#20; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18555,7 +18559,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18601,7 +18605,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18647,7 +18651,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18689,7 +18693,7 @@
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18731,7 +18735,7 @@
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18773,7 +18777,7 @@
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18815,7 +18819,7 @@
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18857,7 +18861,7 @@
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18899,7 +18903,7 @@
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18941,7 +18945,7 @@
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -18983,7 +18987,7 @@
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19025,7 +19029,7 @@
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19067,7 +19071,7 @@
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19109,7 +19113,7 @@
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19151,7 +19155,7 @@
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19177,16 +19181,16 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>R-03</t>
+          <t>R-03 (corregido)</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -19194,10 +19198,14 @@
           <t>US0213M2-P1 (completo)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-03 corregido por MANI-Node#49; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19223,16 +19231,16 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>R-03</t>
+          <t>R-03 (corregido)</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -19240,10 +19248,14 @@
           <t>US0213M2-P1 (parcial)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-03 corregido por MANI-Node#49; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19285,7 +19297,7 @@
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19331,7 +19343,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19373,7 +19385,7 @@
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19415,7 +19427,7 @@
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19457,7 +19469,7 @@
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19499,7 +19511,7 @@
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19541,7 +19553,7 @@
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19583,7 +19595,7 @@
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19625,7 +19637,7 @@
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19667,7 +19679,7 @@
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19709,7 +19721,7 @@
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19751,7 +19763,7 @@
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19793,7 +19805,7 @@
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19835,7 +19847,7 @@
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19889,7 @@
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19919,7 +19931,7 @@
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -19945,16 +19957,16 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>403</v>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+        <v>200</v>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>R-02</t>
+          <t>R-02 (corregido)</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -19962,10 +19974,14 @@
           <t>US0223-P1 (parcial)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-02 corregido por MANI-Node#50 y MANI-.NET#11; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20103,7 +20119,7 @@
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20145,7 +20161,7 @@
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/newman_resumen_20261020T224842Z.json (corrida 20261020T224842Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/newman_resumen_20261021T161015Z.json (corrida 20261021T161015Z)</t>
         </is>
       </c>
     </row>
@@ -20189,7 +20205,7 @@
       <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20233,7 +20249,7 @@
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20277,7 +20293,7 @@
       <c r="I83" s="2" t="inlineStr"/>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20321,7 +20337,7 @@
       <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20365,7 +20381,7 @@
       <c r="I85" s="2" t="inlineStr"/>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20409,7 +20425,7 @@
       <c r="I86" s="2" t="inlineStr"/>
       <c r="J86" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20439,14 +20455,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -20454,10 +20470,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-04 mitigado en QA: /opt/mani monta flutter.env.qa en assets/.env; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20487,14 +20507,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>Fallido</t>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>R-04</t>
+          <t>R-04 (mitigado en QA)</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
@@ -20502,10 +20522,14 @@
           <t>sin equivalente en SCRUM-1264</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>Fallaba el 20 de octubre. R-04 mitigado en QA: /opt/mani monta flutter.env.qa en assets/.env; aprobado en QA el 21 de octubre.</t>
+        </is>
+      </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20549,7 +20573,7 @@
       <c r="I89" s="2" t="inlineStr"/>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20593,7 +20617,7 @@
       <c r="I90" s="2" t="inlineStr"/>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20637,7 +20661,7 @@
       <c r="I91" s="2" t="inlineStr"/>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/playwright_resultados_20261020T224932Z.json (corrida 20261020T224932Z)</t>
+          <t>qa/regresion_sprint4/evidencia/20261021_validacion/playwright_resultados_20261021T170129Z.json (corrida 20261021T170129Z)</t>
         </is>
       </c>
     </row>
@@ -20793,7 +20817,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -20853,7 +20877,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>MANI-docs qa/monitoreo_qas/evidencia/20261020T020546Z_d02/confirmacion_d02_login_real.txt; MANI-Node release src/routes/auth.routes.js:9 (ALLOWED_ALGORITHMS = HS256)</t>
+          <t>MANI-docs qa/monitoreo_qas/evidencia/20261020T020546Z_d02/confirmacion_d02_login_real.txt; MANI-Node release src/routes/auth.routes.js:9 (ALLOWED_ALGORITHMS = HS256). Verificación del 21 oct: MANI-Node#52 y MANI-.NET#13 (develop); MANI-Node#53 y MANI-.NET#14 (release). Login real ES256 con 200 (login_real_es256_20261021T164543Z.txt) y tokens ES256 falsificados con 401 (es256_negativos_20261021.txt). ADR-0031 en MANI-docs#59, abierto.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -20895,7 +20919,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Mitigado en QA (21 oct); corrección en el repositorio pendiente</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -20955,7 +20979,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>playwright_resultados.json; flutter_login_qa.png; MANI-Flutter release .github/workflows/docker-publish.yml:30</t>
+          <t>playwright_resultados.json; flutter_login_qa.png; MANI-Flutter release .github/workflows/docker-publish.yml:30. Verificación del 21 oct: En /opt/mani se monta flutter.env.qa en assets/.env (cambio manual, sin versionar). Playwright FW-02 y FW-03 aprueban (playwright_resultados_20261021T170129Z.json). MANI-Flutter sigue copiando .env.example al construir la imagen.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -21057,7 +21081,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Sin evidencia versionada</t>
+          <t>Sin evidencia versionada. Verificación del 21 oct: El 21 oct se sumó el montaje manual de flutter.env.qa (R-04) al compose sin versionar de /opt/mani.</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -21099,7 +21123,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -21159,7 +21183,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release src/routes/legal.routes.js:7; nginx.conf sin la ruta</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release src/routes/legal.routes.js:8; nginx.conf sin la ruta. Verificación del 21 oct: MANI-APIGateway#20 (develop) y #21 (release). Newman 856-05 en 200 (newman_resumen_20261021T161015Z.json).</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -21201,7 +21225,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -21261,7 +21285,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release GetSiteRulesForAllyUseCase.js:8</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release GetSiteRulesForAllyUseCase.js:45-51. Verificación del 21 oct: MANI-Node#50 y MANI-.NET#11 (develop); MANI-Node#51 y MANI-.NET#12 (release). Newman 853-04 en 200.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -21303,7 +21327,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Abierto en Jira</t>
+          <t>Corregido y verificado en QA (21 oct)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -21363,7 +21387,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release SupabaseDocumentoKycRepository.js:44</t>
+          <t>newman_resumen_20261020T224842Z.json (se reproduce igual que en 20261020T212453Z); MANI-Node release SupabaseDocumentoKycRepository.js:44. Verificación del 21 oct: MANI-Node#49 (develop) y #51 (release). Newman 1066-01 y 1066-02 en 200.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -21405,7 +21429,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -21465,7 +21489,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuario de Core); qa/regresion_sprint4/evidencia/dispatch_rol_20261020T232719Z.txt (usuario de Dispatch)</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 3 y usuario de Core); qa/regresion_sprint4/evidencia/dispatch_rol_20261020T232719Z.txt (usuario de Dispatch). Verificación del 21 oct: consultas_rls_20261021T170441Z.txt (Core y Dispatch)</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -21507,7 +21531,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -21567,7 +21591,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>newman_reporte_redactado_20261020T224842Z.json (cuerpos de 862-02, 1074-03 y 1074-04; igual en newman_reporte_redactado.json de 20261020T212453Z)</t>
+          <t>newman_reporte_redactado_20261020T224842Z.json (cuerpos de 862-02, 1074-03 y 1074-04; igual en newman_reporte_redactado.json de 20261020T212453Z). Verificación del 21 oct: Cuerpos de 862-02 y 1074-04 en newman_reporte_redactado_20261021T161015Z.json</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -21609,7 +21633,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -21669,7 +21693,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (secciones 1, 1b y 1c)</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (secciones 1, 1b y 1c). Verificación del 21 oct: consultas_rls_20261021T170441Z.txt</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -21711,7 +21735,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Abierto (reverificado 21 oct)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -21771,7 +21795,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 2); qa/regresion_sprint4/evidencia/verify_0007_rls_20261020T202905Z.log</t>
+          <t>qa/regresion_sprint4/evidencia/consultas_rls_20261020T225146Z.txt (sección 2); qa/regresion_sprint4/evidencia/verify_0007_rls_20261020T202905Z.log. Verificación del 21 oct: consultas_rls_20261021T170441Z.txt</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -22127,17 +22151,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Toda la regresión usó tokens HS256 sintéticos firmados con el JWT secret legado de MANI-QA. Un usuario real recibe un token ES256 que el Gateway rechaza (R-10, comprobado en SCRUM-1266). Los usuarios de prueba que SCRUM-1269 prevé no se pueden usar mientras R-10 siga abierto.</t>
+          <t>La regresión sigue usando tokens HS256 sintéticos, válidos mientras la clave HS256 legada de MANI-QA no se revoque. Desde el 21 oct un usuario real sí usa las rutas protegidas (R-10 corregido): login de admin.t1 con token ES256 y 200 en Core y Rules; Dispatch acepta el token (login_real_es256_20261021T164543Z.txt). Solo se verificó con ese usuario y esas tres rutas.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Desarrollo (R-10)</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22208,7 +22232,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>No se ejecutaron flujos de interfaz: la web de QA usa el Supabase de producción (R-04) y, aunque se corrija, un usuario real no puede usar rutas protegidas (R-10).</t>
+          <t>No se ejecutaron flujos de interfaz. Desde el 21 oct R-04 está mitigado en QA y R-10 corregido, así que ya no los bloquean: la suite Playwright no tiene todavía flujos Flutter Web → Gateway → servicios.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -22218,7 +22242,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>DevOps y Desarrollo</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22235,7 +22259,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>B4-01 borra una ausencia inexistente y solo es un control; el borrado ajeno se prueba en 855-04. B6 se ejecutó sobre el detalle de verificación de otro tenant; las URL firmadas de Storage no se probaron (R-03).</t>
+          <t>B4-01 es un control con un id inexistente; el borrado ajeno se prueba en 855-04. B6 no cubre las URL firmadas de Storage: R-03, que lo impedía, está corregido desde el 21 oct, pero el caso no se ha ejecutado.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -22245,7 +22269,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Prueba de QA</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
@@ -22316,7 +22340,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Habilitado por QA el 20 de octubre y ejecutado una vez (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 77 solicitudes, 125 aserciones y 5 fallidas; Playwright 11 pruebas y 9 aprobadas. Los dos jobs quedan en rojo por R-01 a R-04 (corrida en rojo del DoD); la corrida en verde depende de esas correcciones. No es check obligatorio de la rama. GOBIERNO_DEL_EQUIPO §2.3 asigna CI/CD y secretos a DevOps.</t>
+          <t>Habilitado por QA el 20 oct y ejecutado en CI una vez (run 39513870492), en rojo por R-01 a R-04 (corrida en rojo del DoD). Tras las correcciones, la regresión del 21 oct en la VM de QA da 0 fallas (Newman 20261021T161015Z y Playwright 20261021T170129Z), pero la corrida en verde en CI no se ha hecho. El gate no es un check obligatorio de la rama. GOBIERNO_DEL_EQUIPO §2.3 asigna CI/CD y secretos a DevOps.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -22343,7 +22367,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>RLS no se ejerce en QA (R-06, R-07 y R-09, con evidencia en consultas_rls_20261020T225146Z.txt). El aislamiento comprobado es el de la aplicación a través del Gateway.</t>
+          <t>RLS no se ejerce en QA (R-06, R-07 y R-09, reverificados el 21 oct en consultas_rls_20261021T170441Z.txt). El aislamiento comprobado es el de la aplicación a través del Gateway.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -22423,7 +22447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22505,53 +22529,65 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Multi-tenant X1 a X6 (SCRUM-1279)</t>
+          <t>Sin ejecutar (historia)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Por caso: aprobado, fallido, bloqueado o no ejecutable, según el DoD de SCRUM-1279; "no aplica" cuando SCRUM-1264 lo declara así y "sin ejecutar" cuando el caso es ejecutable y QA no lo corrió. "(parcial)" indica que el caso de regresión cubre una parte del caso diseñado.</t>
+          <t>La historia ya no tiene bloqueo externo y QA no ha ejecutado sus casos. No es un estado del vocabulario de SCRUM-1267: se declara para no ocultar la brecha (usado en SCRUM-1060 desde el 21 de octubre).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Cobertura de un caso de SCRUM-1264</t>
+          <t>Multi-tenant X1 a X6 (SCRUM-1279)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>completo: un caso válido verifica lo que pide el caso diseñado; parcial: verifica una parte; sin ejecutar: ningún caso válido lo cubre.</t>
+          <t>Por caso: aprobado, fallido, bloqueado o no ejecutable, según el DoD de SCRUM-1279; "no aplica" cuando SCRUM-1264 lo declara así y "sin ejecutar" cuando el caso es ejecutable y QA no lo corrió. "(parcial)" indica que el caso de regresión cubre una parte del caso diseñado.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Caso no válido, no concluyente o excluido</t>
+          <t>Cobertura de un caso de SCRUM-1264</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>No cuenta como evidencia (ver la nota del caso).</t>
+          <t>completo: un caso válido verifica lo que pide el caso diseñado; parcial: verifica una parte; sin ejecutar: ningún caso válido lo cubre.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Caso no válido, no concluyente o excluido</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>No cuenta como evidencia (ver la nota del caso).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Origen</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Desarrollo: la prueba sigue el criterio o el contrato y el sistema responde distinto. DevOps: el mismo código funciona con otra configuración o falta un componente del despliegue. QA: la prueba, los datos o la cobertura no corresponden al criterio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22589,7 +22625,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-20 (regresión) y 2026-10-21 (validación de las correcciones)</t>
         </is>
       </c>
     </row>
@@ -22601,7 +22637,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>QA 10.43.100.141 (release; Gateway 82473d6, Core 2745bb0, Rules e90f32b, Dispatch 41ba171, Flutter 74bab53, Landing a82b94e; base Supabase MANI-QA)</t>
+          <t>QA 10.43.100.141, rama release, base Supabase MANI-QA. Desde el redespliegue del 21 oct: Gateway f042817, Core 8ad4a35, Rules e90f32b, Dispatch 0998a3d, Flutter 8e606e4 y Landing a82b94e, iguales a la cabeza de release (ambiente_qa_20261021.txt). El 20 oct: Gateway 82473d6, Core 2745bb0, Dispatch 41ba171 y Flutter 74bab53.</t>
         </is>
       </c>
     </row>
@@ -22625,7 +22661,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tokens HS256 sintéticos firmados en la VM con el JWT secret legado de MANI-QA (L-01, R-10)</t>
+          <t>Tokens HS256 sintéticos firmados en la VM con el JWT secret legado de MANI-QA (L-01). Desde el 21 oct, login real con ES256 verificado para admin.t1 (R-10 corregido).</t>
         </is>
       </c>
     </row>
@@ -22637,7 +22673,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Compose, .env.qa y recreación de contenedores: QA (Santiago Hernández). Migraciones de Core 0001-0010 y 0013 aplicadas por QA desde el SQL Editor de MANI-QA. Respaldo previo en /opt/mani. Según GOBIERNO_DEL_EQUIPO §2.3 estas decisiones corresponden a DevOps; comunicación formal a DevOps pendiente.</t>
+          <t>Compose, .env.qa y recreación de contenedores: QA (Santiago Hernández). Migraciones de Core 0001-0010 y 0013 aplicadas por QA desde el SQL Editor de MANI-QA. Respaldo previo en /opt/mani. Según GOBIERNO_DEL_EQUIPO §2.3 estas decisiones corresponden a DevOps; comunicación formal a DevOps pendiente. El 21 oct, QA agregó al compose de /opt/mani el montaje de flutter.env.qa en assets/.env de flutter-web (R-04, con autorización de Santiago Hernández y respaldo previo); queda para que DevOps lo valide en el despliegue.</t>
         </is>
       </c>
     </row>
@@ -22649,7 +22685,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Vigentes: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida). Anteriores: Newman 20261020T212453Z y Playwright 20261020T212519Z. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z. Gate de CI desde el runner de Calidad (run 39513870492 de MANI-APIGateway (https://github.com/Trama-AS/MANI-APIGateway/actions/runs/39513870492)): Newman 20261020T234635Z y Playwright 20261020T235520Z.</t>
+          <t>Vigentes (21 oct, tras las correcciones): Newman 20261021T161015Z y Playwright 20261021T170129Z. Del 20 oct: Newman 20261020T224842Z y Playwright 20261020T224932Z (colección corregida), Newman 20261020T212453Z y Playwright 20261020T212519Z (primera corrida) y gate de CI run 39513870492. Consultas de solo lectura sobre MANI-QA: 20261020T225146Z y 20261021T170441Z.</t>
         </is>
       </c>
     </row>

</xml_diff>